<commit_message>
Updated NGA_grids_kan model - 2025-12-05 16:28
</commit_message>
<xml_diff>
--- a/VerveStacks_NGA_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NGA_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NGA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8EF3B14-9273-4BD6-A37D-01982B1A002A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B116DB73-3C33-4455-BCB7-4032B2FDA50B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24578,7 +24578,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15E6F76F-AA31-4310-B232-F900661E6B29}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{794CAA10-11EA-4364-937F-D9B0D7A76A85}">
   <dimension ref="B9:H145"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27316,7 +27316,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D56BB41-E9F4-48A9-BB44-63EDF3928C1C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1BCACFE-A23F-4E23-A884-CA3C6C9432E6}">
   <dimension ref="B9:L145"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NGA_grids_kan model - 2025-12-05 21:34
</commit_message>
<xml_diff>
--- a/VerveStacks_NGA_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NGA_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NGA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B116DB73-3C33-4455-BCB7-4032B2FDA50B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B5F88A9-FBCA-41F6-B108-BF7FE5A10481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24578,7 +24578,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{794CAA10-11EA-4364-937F-D9B0D7A76A85}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0138AFE7-544F-41FE-BD3C-380014FB1A8F}">
   <dimension ref="B9:H145"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27316,7 +27316,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1BCACFE-A23F-4E23-A884-CA3C6C9432E6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0D089EA-DA44-42D6-94D7-5FF8F138B66A}">
   <dimension ref="B9:L145"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NGA_grids_kan model - 2025-12-06 14:26
</commit_message>
<xml_diff>
--- a/VerveStacks_NGA_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NGA_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NGA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{96BDD199-9496-4C03-A739-FA4365C0BA1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADB1C9C5-A807-4F4D-87E3-D6555A7E9918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24578,7 +24578,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{968A3CF8-471D-402F-B706-4A6B04C21177}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AAA184C-307E-4BEE-B478-DCAE902B6D29}">
   <dimension ref="B9:H145"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -27316,7 +27316,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{132F03D2-DD83-40E9-A246-CA00D7A1F898}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FB9DB41-6DC9-4049-91DA-BC0D52F1BEB3}">
   <dimension ref="B9:L145"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated NGA_grids_kan model - 2025-12-12 14:02
</commit_message>
<xml_diff>
--- a/VerveStacks_NGA_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_NGA_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NGA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA1A6AB4-3624-42D3-B442-A54D5249DA2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B96AD263-768F-4677-98D6-75F4ADA15286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3340,7 +3340,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB33D683-33F5-40E1-9503-C46345F64118}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70F70D5C-7E83-49BD-9DBA-671211EB6DC2}">
   <dimension ref="B9:H145"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -22557,7 +22557,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28C43500-B4C7-4EA5-8CC8-66ED43B0A11D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB24B721-A272-438A-8E4C-C9B44FAD93BA}">
   <dimension ref="B9:L145"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>